<commit_message>
fixed CAPE scoring remaining bugs
now works as intended, see wiki backbone scoring for details
</commit_message>
<xml_diff>
--- a/information/2025-10-28_Scoring.xlsx
+++ b/information/2025-10-28_Scoring.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Wilken_Arbeitsordner\Clinical_Backbone_RU5389\information\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37C207F3-763A-4510-8498-252CAA6C0BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E4956CF-A395-4A0F-9209-DD221431849C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="27">
   <si>
     <t>IDAS</t>
   </si>
@@ -100,9 +100,6 @@
   </si>
   <si>
     <t>scale</t>
-  </si>
-  <si>
-    <t>mean(distress * frequency)</t>
   </si>
   <si>
     <t>sum(agree)</t>
@@ -433,14 +430,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" width="25.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="65.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="65.453125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="209" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -460,7 +457,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -477,24 +474,24 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D3" t="s">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="F3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -505,18 +502,18 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E5" t="s">
         <v>11</v>
@@ -525,7 +522,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -542,7 +539,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -553,13 +550,13 @@
         <v>4</v>
       </c>
       <c r="D7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -576,7 +573,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -596,7 +593,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -613,7 +610,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -630,7 +627,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -647,7 +644,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>21</v>
       </c>

</xml_diff>